<commit_message>
dong bo hoan toan dac ta v0 va v1: 10 sheet excel, 28 test cases, 7 ham sinh ma va 6 phep kiem tra z3
</commit_message>
<xml_diff>
--- a/01_spec/quanly_khohang_v1.xlsx
+++ b/01_spec/quanly_khohang_v1.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -562,444 +562,1060 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>TC-01</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>REQ-01, CON-01</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>H1: Nạp chuỗi 32 và 33 byte bị từ chối an toàn</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>ingest_raw_line_v1 có rào chắn kiểm tra len &lt; 32 - M1 Thọ</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Gọi ingest_raw_line_v1 với chuỗi dài 32 và 33 ký tự</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Hàm từ chối xử lý, trả về mã lỗi an toàn -2, 0 byte bị ghi đè</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC-M1-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>REQ-1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Nạp dòng chuỗi chuẩn độ dài ngắn (len = 15 &lt; 32 bytes) vào buffer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Chuỗi raw_line hợp lệ: SP001;GaoST25;100;25000 (23 bytes)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Khởi tạo buffer stack 32 byte
+Thực hiện nạp chuỗi raw_line vào buffer</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>v0 và v1 đều nạp chuỗi thành công, buffer nhận đúng nội dung</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>TC-02</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>REQ-02, CON-01</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>H1: Nạp chuỗi hợp lệ 31 byte thành công</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>char buffer[32], cap = 32, chuỗi dài 31 ký tự - M1 Thọ</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Gọi ingest_raw_line_v1 với chuỗi 31 byte</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Trả về 31, sao chép thành công và kết thúc bằng '\0'</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC-M1-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>REQ-1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nạp dòng chuỗi cận trên an toàn (len = 31 bytes có null-terminator)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Chuỗi raw_line dài chính xác 31 ký tự + 1 byte null = 32 byte</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Khởi tạo buffer stack 32 byte
+Nạp chuỗi biên 31 byte vào buffer</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>v0 và v1 đều sao chép an toàn, ký tự kết thúc chuỗi '\0' được bảo toàn</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>TC-03</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>REQ-03, CON-02</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>H2: Đọc token ngoài biên bị từ chối có kiểm soát</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>token_count = 4, field_idx = 4 hoặc field_idx = -1 - M1 Thọ</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Gọi get_token_field_v1 với chỉ số ngoài biên</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Rào chắn phát hiện chỉ số vi phạm, từ chối an toàn trả về -2</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC-M1-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>REQ-2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Đọc trường token đầu tiên (field_idx = 0) từ danh sách token hợp lệ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mảng token đã phân tách gồm 4 trường SP001, GaoST25, 100, 25000 (token_count = 4)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Gọi hàm get_token_field với field_idx = 0
+Lấy giá trị mã hàng</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Truy xuất thành công trường mã hàng SP001, không lỗi</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TC-04</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>REQ-04, CON-02</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>H2: Đọc token với con trỏ mảng NULL</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>token_offsets = NULL - M1 Thọ</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Gọi get_token_field_v1 với con trỏ NULL</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Rào chắn phát hiện mảng NULL, trả về -1</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC-M1-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>REQ-2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Đọc trường token cuối cùng (field_idx = token_count - 1)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>token_count = 4, truy xuất trường đơn giá tại chỉ số 3</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Gọi hàm get_token_field với field_idx = 3
+Lấy giá trị đơn giá</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Truy xuất thành công trường đơn giá 25000</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TC-05</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>REQ-05, CON-03</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>H3: OOM khi realloc bảo toàn vùng nhớ cũ</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>mock_realloc trả về NULL - M2 Trang</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Gọi expand_stock_items_v1 khi hết RAM</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Bảo toàn 100% con trỏ cũ qua biến tạm tmp, trả về STATUS_ERR_ALLOC</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC-M1-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>REQ-3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Kiểm toán an toàn chu trình I/O toàn diện không vi phạm bộ nhớ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Chạy qua toàn bộ chu trình nạp chuỗi và đọc token</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Kiểm tra bất biến AG(!violation) trên toàn bộ không gian trạng thái</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>v0: Vi phạm an toàn (CWE-120/125); v1: Thỏa mãn 100% AG(!violation)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TC-06</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>REQ-06, CON-03</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>H3: Kích thước mở rộng được chặn cận trên</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>new_capacity vượt giới hạn an toàn - M2 Trang</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Kiểm tra SMT Z3 trên heap_alloc_bytes</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Z3 chứng minh UNSAT: không tồn tại nghiệm vi phạm</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC-M1-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Kích hoạt lỗi tràn bộ đệm stack với chuỗi dữ liệu vượt ngưỡng (len = 64 bytes)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Chuỗi raw_line chứa 64 ký tự (vượt quá stack buffer 32 byte)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Gọi ingest_raw_line với chuỗi 64 byte
+Quan sát vùng nhớ stack liền kề</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>v0: Ghi đè frame stack và con trỏ trả về (CWE-120/121); v1: Chặn từ chối an toàn do len &gt;= 32</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>REQ-07, CON-04</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>H4: Rào chắn ngăn chặn tràn số cộng dồn</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>current_stock = 2.147.483.640, added_quantity = 20 - M3 Đô</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Gọi update_stock_quantity_v1</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Phát hiện nguy cơ tràn số trước khi thực hiện, trả về ERR_OVERFLOW</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC-M1-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bắt lỗi Off-by-one khi chuỗi có đúng 32 byte dữ liệu thiếu null-terminator</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Chuỗi đầu vào có đúng 32 ký tự, không còn chỗ cho ký tự null kết thúc chuỗi</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sao chép 32 byte vào buffer[32] bằng strcpy
+Đọc chuỗi sau khi sao chép</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>v0: Đọc tràn qua biến tiếp theo trên stack do thiếu null (CWE-193); v1: buffer[31] = '\0'</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>REQ-08, CON-04</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>H4: Từ chối số lượng nhập hàng âm</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity = -50 - M3 Đô</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Gọi update_stock_quantity_v1 với số âm</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Từ chối an toàn trả về ERR_NEGATIVE</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-M1-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Phát hiện lỗi Stack Buffer Overflow bằng AddressSanitizer (ASan Crash Trigger)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Biên dịch mã nguồn C với flag -fsanitize=address</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Thực thi hàm ingest_raw_line với chuỗi 48 ký tự
+Ghi nhận cảnh báo từ ASan</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>v0: ASan báo lỗi ERROR: AddressSanitizer: stack-buffer-overflow; v1: 0 crash</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>TC-09</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>REQ-09, CON-04</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>H5: Rào chắn ngăn chặn tràn phép nhân đơn giá</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>base_price lớn và rate lớn - M3 Đô</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Gọi scale_product_price_v1</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Kiểm tra base_price &gt; INT_MAX / rate, từ chối an toàn</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-M1-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bắt lỗi đọc ngoài biên mảng token khi chỉ số vượt trần (field_idx &gt;= token_count)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>token_count = 4, yêu cầu đọc trường tại field_idx = 4 hoặc field_idx = 10</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Gọi get_token_field(4, 4)
+Kiểm tra con trỏ token trả về</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>v0: Đọc ngoài biên mảng con trỏ token (CWE-125); v1: Phát hiện và trả về NULL/mã lỗi an toàn</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TC-10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>REQ-10, CON-05</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>H6: Mutex đồng bộ hoàn toàn giữa 2 worker</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Cả 2 worker truy cập phiên kho - M2 Trang</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Kiểm tra loại trừ lẫn nhau trên Kripke v1</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Thỏa mãn 100%, 0 vi phạm tranh chấp</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-M1-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Bắt lỗi đọc ngoài biên mảng token khi chỉ số âm (field_idx = -1 &lt; 0)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Yêu cầu đọc trường với chỉ số âm field_idx = -1</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Gọi get_token_field(4, -1)
+Kiểm tra phản hồi của hệ thống</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>v0: Đọc vùng nhớ phía trước mảng token (CWE-125); v1: Chặn ngay tại điều kiện field_idx &lt; 0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TC-11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>REQ-11, REQ-12</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>H6: Con trỏ được gán NULL ngay sau free</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Gọi release_stock_items_v1 - M2 Trang</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Kiểm tra con trỏ sau khi free()</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>list == NULL, triệt tiêu hoàn toàn lỗi Use-After-Free và Double-Free</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-M1-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>REQ-6</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Kiểm tra tính sống: Không xảy ra deadlock trong toàn bộ chu trình xử lý I/O</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Mô hình chuyển trạng thái Kripke của module M1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Duyệt qua tất cả 7 trạng thái
+Kiểm tra bậc ra out-degree của từng trạng thái</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Mọi trạng thái đều có out-degree &gt;= 1, 0 deadlock, công thức AF(done) thỏa mãn trên v1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TC-12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>REQ-01 đến REQ-12</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Kiểm chứng toàn luồng quản lý kho an toàn v1</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Mô hình kết hợp 27 trạng thái bản v1</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Chạy chay_kiem_chung_kripke.py</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Không deadlock, 100% 18 công thức CTL THỎA MÃN</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-M1-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>REQ-1, REQ-2, REQ-3, REQ-4, REQ-5, REQ-6</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Kiểm thử hồi quy đối chứng toàn diện pytest (Regression Verification Suite)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Bộ test pytest tự động test_verify_v0_cases_on_v1.py</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Chạy kiểm thử toàn bộ test cases trên bản v0
+Chạy kiểm thử toàn bộ test cases trên bản v1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>v0: Bắt đầy đủ lỗi CWE-120/121, CWE-193, CWE-125; v1: 100% PASSED</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC-M2-01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>REQ-1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Khởi tạo mảng động danh mục hàng ban đầu (Initial Capacity)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Khởi tạo danh sách rỗng product_list_init(&amp;list)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Gọi hàm khởi tạo danh mục
+Kiểm tra count == 0, capacity == 16, con trỏ items != NULL</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Thành công: Cấp phát đúng 16 ô nhớ ban đầu trên Heap</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC-M2-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>REQ-1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Thêm sản phẩm tới chạm ngưỡng dung lượng chưa mở rộng (Fill to Capacity)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Danh sách đang có capacity = 16</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Thêm liên tiếp 16 sản phẩm hợp lệ vào danh sách
+Kiểm tra count == 16, capacity == 16</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Thành công: 16 sản phẩm được lưu trọn vẹn, chưa kích hoạt realloc</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC-M2-03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>REQ-1, REQ-6</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Tự động nhân đôi dung lượng khi thêm sản phẩm thứ 17 (Capacity Doubling)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Danh sách đã đầy 16 phần tử, thêm phần tử thứ 17</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Gọi add_product thêm sản phẩm thứ 17
+Kiểm tra capacity tăng từ 16 lên 32, count == 17</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Thành công: Thuật toán nhân đôi mảng động cấp phát vùng nhớ mới an toàn</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC-M2-04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>REQ-6</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Kiểm tra tràn số nguyên khi tính toán kích thước mở rộng (Integer Overflow in Capacity)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>current_capacity vượt ngưỡng an toàn (ví dụ: SIZE_MAX / 2)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Chạy kiểm tra SMT Z3 trên điều kiện heap_alloc_bytes
+Thực thi hàm calc_expand_capacity_v0 với factor lớn</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>v0: Phép nhân tràn số âm/nhỏ gây cấp phát thiếu ô nhớ; v1: Rào chắn từ chối mở rộng</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC-M2-05</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Mô phỏng sự cố OOM khi realloc mảng động (Fault Injection OOM NULL)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Hệ thống cạn kiệt RAM, mock_realloc trả về NULL</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Ép hàm realloc trả về NULL khi mảng đầy cần mở rộng
+Quan sát phản ứng của hàm mở rộng</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>v0: Gán list = NULL làm mất sạch địa chỉ vùng nhớ cũ; v1: Trả về STATUS_ERR_ALLOC</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TC-M2-06</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Bảo toàn địa chỉ và quyền sở hữu vùng nhớ cũ khi OOM (Ownership Retention)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>realloc trả về NULL</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>So sánh địa chỉ con trỏ items trước và sau khi realloc thất bại</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>v0: Con trỏ gốc bị ghi đè thành NULL; v1: Địa chỉ cũ được bảo toàn 100%</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TC-M2-07</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Bảo toàn tính toàn vẹn của dữ liệu đã có khi OOM (Data Integrity on Failure)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Danh sách chứa sẵn 16 mặt hàng ban đầu</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sau khi mở rộng thất bại, duyệt đọc lại 16 mặt hàng cũ</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>v0: Crash bộ nhớ do con trỏ bị NULL hóa; v1: 16 mặt hàng cũ còn nguyên vẹn</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC-M2-08</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Kiểm toán rò rỉ bộ nhớ bằng LeakSanitizer (LSan Memory Leak Audit)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Biên dịch bản v0 và v1 với flag -fsanitize=leak</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Chạy kịch bản nhập kho OOM trên bản v0 và v1
+Kiểm tra log của LeakSanitizer</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>v0: LSan bắt lỗi leaked 16 blocks (CWE-401); v1: LSan báo 0 byte leaked</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TC-M2-09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Con trỏ mượn bị vô hiệu hóa sau khi mảng động dời địa chỉ (Dangling Pointer on Resize)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Lưu con trỏ mượn p = find_product_by_id(&amp;list, "P0001")</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Gọi add_product kích hoạt realloc sang địa chỉ RAM mới
+Đọc dữ liệu qua con trỏ p ban đầu</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>v0: p trỏ vào vùng nhớ cũ đã bị OS thu hồi; v1: Cảnh báo Borrowed Pointer Invalidation</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TC-M2-10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Đọc con trỏ sau khi free phiên kho (Use-After-Free Audit)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Hàm cleanup_and_read_uaf_v0 giải phóng struct nhưng vẫn return *ptr</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Gọi hàm giải phóng tài nguyên phiên kho
+Thực hiện đọc/ghi vào con trỏ vừa giải phóng</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>v0: Đọc dữ liệu rác/vùng nhớ tự do (CWE-416); v1: Triệt tiêu hoàn toàn vì con trỏ đã set NULL</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TC-M2-11</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Bắt lỗi Heap-Use-After-Free bằng AddressSanitizer (ASan Crash Trigger)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Biên dịch mã nguồn với flag -fsanitize=address</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Thực thi test_sim001_heap trên bản v0
+Ghi nhận crash log do ASan sinh ra</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>v0: ASan sinh log crash: ERROR: AddressSanitizer: heap-use-after-free on address; v1: 0 crash</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TC-M2-12</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Phòng thủ giải phóng hai lần trên cùng một con trỏ (Double-Free Defense)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Gọi product_list_free(&amp;list) liên tiếp 2 lần</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Thực hiện lệnh free(list-&gt;items) lần 1
+Thực hiện tiếp lệnh free(list-&gt;items) lần 2</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>v0: Crash OS double free or corruption (CWE-415); v1: Lần 2 gặp con trỏ NULL nên bỏ qua an toàn</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TC-M2-13</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>REQ-3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Kiểm toán bất biến an toàn bộ nhớ (Safety Invariant: count &lt;= capacity)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Chạy qua 50 lần thêm/xóa ngẫu nhiên</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Kiểm tra điều kiện list.count &lt;= list.capacity tại mọi thời điểm</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Bất biến an toàn luôn được duy trì 100% trong suốt vòng đời mảng động</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TC-M2-14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>REQ-1, REQ-2, REQ-3, REQ-4, REQ-5</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Kiểm thử hồi quy đối chứng toàn diện pytest (Regression Verification Suite)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Bộ test pytest test_verify_v0_cases_on_v1.py</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Chạy toàn bộ test cases trên bản lỗi v0
+Chạy lại toàn bộ test cases trên bản vá v1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>v0: Phát hiện đầy đủ lỗi CWE-190, CWE-401, CWE-416; v1: 100% PASSED (Xanh toàn bộ)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TC-M3-01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>REQ-1, REQ-4</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Cộng dồn số lượng hàng hóa gây tràn số nguyên có dấu 32-bit</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>old_stock = 2.147.483.640, added_quantity = 100</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Chạy check_satisfiability() trên stock_addition_overflow (Chương 3 Z3)
+Kiểm tra AG(!integer_overflow) trên luồng M3-v0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>v0: VI PHẠM (CWE-190 Signed Integer Overflow), kết quả lật âm; v1: ĐÚNG (chặn trước khi cộng)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TC-M3-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>REQ-3, REQ-5</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Từ chối số lượng nhập hàng là số âm</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>added_quantity = -50</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Kiểm tra AG(!negative_input) trên luồng M3-v0
+Kiểm tra lại trên luồng M3-v1</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>v0: VI PHẠM (nhận số âm); v1: ĐÚNG (rào chắn từ chối ngay lập tức)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2798,225 +3414,190 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ingest_raw_line</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>buffer_copy</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>dst, cap, raw_line</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>raw_line</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>32</v>
       </c>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>H1 — Nạp chuỗi an toàn phòng thủ (M1 Thọ)</t>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>H1 — Nạp chuỗi an toàn phòng thủ strncpy/giới hạn 32 byte (M1 Thọ)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>get_token_field</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>array_read</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>token_offsets, token_count, field_idx</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>H2 — Đọc token an toàn phòng thủ (M1 Thọ)</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>arithmetic</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>token_count, field_idx</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>H2 — Kiểm tra biên token an toàn [0, token_count-1] (M1 Thọ)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>expand_stock_items</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>alloc_release</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>list, new_capacity</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>16</v>
       </c>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>H3 — realloc an toàn bảo toàn vùng nhớ qua tmp (M2 Trang)</t>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>H3 — Cấp phát Heap và giải phóng an toàn free(buf) (M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>release_stock_items</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>alloc_release</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>list</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" t="n">
         <v>16</v>
       </c>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>H6 — free() và gán con trỏ = NULL (M2 Trang)</t>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>H6 — free() xong gán buf = NULL triệt tiêu UAF (M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>update_stock_quantity</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>arithmetic</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>current_stock, added_quantity</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>H4 — Cộng tồn kho an toàn phòng thủ (M3 Đô)</t>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>H4 — Cộng dồn tồn kho có rào chắn chặn tràn INT_MAX (M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>scale_product_price</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>arithmetic</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>base_price, rate</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>H5 — Nhân tỉ giá an toàn phòng thủ (M3 Đô)</t>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>H5 — Nhân tỉ giá có rào chắn chặn tràn int32 (M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>calc_batch_capacity</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>python</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>divide</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>total_items, batch_size</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>H3 — Kiểm tra batch_size &gt; 0 trước khi chia</t>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>H3 — Kiểm tra batch_size != 0 trước khi chia (M2 Trang)</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3069,110 +3650,164 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>buffer_capacity_check</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>cap, input_len</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>cap == 32 and input_len &lt; cap</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>input_len - cap</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>H1 — Rào chắn kiểm tra độ dài input_len &lt; 32 byte ngăn chặn tràn stack (M1 Thọ - Z3 UNSAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>token_index_check</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>token_count, field_idx</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>token_count &gt; 0 and (field_idx &lt; 0 or field_idx &gt;= token_count)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>field_idx - token_count</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>H2 — Rào chắn từ chối chỉ số âm hoặc vượt trần (M1 Thọ - Z3 UNSAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>heap_alloc_bytes</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>new_capacity, item_size</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>new_capacity &gt;= 1 and item_size == 48 and new_capacity * item_size &gt; 2147483647</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>new_capacity * item_size</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>H3 — Rào chắn MAX_SAFE_CAPACITY ngăn chặn tràn Heap (M2 Trang - Z3 UNSAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>stock_addition_overflow</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>current_stock, added_quantity</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>current_stock &gt;= 0 and added_quantity &gt;= 1 and current_stock + added_quantity &gt; 2147483647</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>current_stock + added_quantity</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>H4 — rào chắn ngăn chặn hoàn toàn (Z3 UNSAT trên v1 - M3 Đô)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>heap_alloc_bytes</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>new_capacity, item_size</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>new_capacity &gt;= 1 and item_size == 48 and new_capacity * item_size &gt; 2147483647</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>new_capacity * item_size</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>H3 — rào chắn giới hạn MAX_SAFE_CAPACITY (Z3 UNSAT - M2 Trang)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>old_stock, added_quantity</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>old_stock &gt;= 0 and old_stock &lt;= 2147483647 and added_quantity &gt;= 1 and added_quantity &lt;= 2147483647 and old_stock + added_quantity &gt; 2147483647</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>old_stock + added_quantity</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>H4 — Rào chắn INT_MAX - added_quantity từ chối trước khi cộng (M3 Đô - Z3 UNSAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>negative_quantity_check</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>added_quantity</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>added_quantity &lt; 0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>added_quantity</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>H4 — Rào chắn từ chối số lượng nhập âm ngay khi nhận (M3 Đô - Z3 UNSAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>price_multiplication_overflow</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>base_price, rate</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>base_price &gt; 0 and rate &gt; 1 and base_price * rate &gt; 2147483647</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>base_price * rate</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>H5 — rào chắn kiểm tra trần nhân (Z3 UNSAT - M3 Đô)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>negative_quantity_check</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity &lt; 0</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>H4 — từ chối số âm trước khi xử lý (Z3 UNSAT - M3 Đô)</t>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>H5 — Rào chắn kiểm tra trần nhân giá x tỉ giá (M3 Đô - Z3 UNSAT)</t>
         </is>
       </c>
     </row>

</xml_diff>